<commit_message>
Created hall effect test script for T4.1, adjusted hall effect input strategy
</commit_message>
<xml_diff>
--- a/PCB/DAQBoardFront/JLCPCB Docs/BOM_DAQ.xlsx
+++ b/PCB/DAQBoardFront/JLCPCB Docs/BOM_DAQ.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a56d338d63da0fa/Desktop/CFR-2027/PCB/DAQBoardFront/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a56d338d63da0fa/Desktop/CFR-2027/PCB/DAQBoardFront/JLCPCB Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="8_{672BEF6D-422F-477B-B486-B83020C6D7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD1300AD-9901-4271-A29F-34D2B4B6F193}"/>
+  <xr:revisionPtr revIDLastSave="80" documentId="8_{672BEF6D-422F-477B-B486-B83020C6D7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EF2B4F8-5DBA-4DC7-9FF7-409359123BDF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{93B5DAD3-BF6B-4E2E-A13F-1D74895200EB}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="78">
   <si>
     <t>Designator</t>
   </si>
@@ -64,18 +64,9 @@
     <t>C_0603_1608Metric</t>
   </si>
   <si>
-    <t>C2, C3</t>
-  </si>
-  <si>
     <t>C_0603_1608Metric_Pad1.08x0.95mm_HandSolder</t>
   </si>
   <si>
-    <t>C4, C5</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
     <t>C6, C7</t>
   </si>
   <si>
@@ -91,9 +82,6 @@
     <t>C_1206_3216Metric_Pad1.33x1.80mm_HandSolder</t>
   </si>
   <si>
-    <t>D2, D3, D4</t>
-  </si>
-  <si>
     <t>SODFL2512X90N</t>
   </si>
   <si>
@@ -109,24 +97,9 @@
     <t>LMR51430YDDCR</t>
   </si>
   <si>
-    <t>J1</t>
-  </si>
-  <si>
-    <t>CONN10_533751010_MOL</t>
-  </si>
-  <si>
     <t>~</t>
   </si>
   <si>
-    <t>J2</t>
-  </si>
-  <si>
-    <t>0533750410</t>
-  </si>
-  <si>
-    <t>53375-0410</t>
-  </si>
-  <si>
     <t>L_0805_2012Metric_Pad1.05x1.20mm_HandSolder</t>
   </si>
   <si>
@@ -145,21 +118,12 @@
     <t>R_0603_1608Metric_Pad0.98x0.95mm_HandSolder</t>
   </si>
   <si>
-    <t>R</t>
-  </si>
-  <si>
-    <t>R4, R7, R9</t>
-  </si>
-  <si>
     <t>LED_0603_1608Metric_Pad1.05x0.95mm_HandSolder</t>
   </si>
   <si>
     <t>24k</t>
   </si>
   <si>
-    <t>R5, R8, R10</t>
-  </si>
-  <si>
     <t>2k</t>
   </si>
   <si>
@@ -178,21 +142,6 @@
     <t>ERJ-3EKF1372V</t>
   </si>
   <si>
-    <t>R13, R14</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>R15</t>
-  </si>
-  <si>
-    <t>R_1206_3216Metric</t>
-  </si>
-  <si>
-    <t>CSR1206FT50L0</t>
-  </si>
-  <si>
     <t>R16, R17</t>
   </si>
   <si>
@@ -214,30 +163,12 @@
     <t>56.2k</t>
   </si>
   <si>
-    <t>T1</t>
-  </si>
-  <si>
-    <t>AC1210-110-C</t>
-  </si>
-  <si>
     <t>T2</t>
   </si>
   <si>
     <t>NCS2005SN1T1G</t>
   </si>
   <si>
-    <t>U1</t>
-  </si>
-  <si>
-    <t>MODULE_2019</t>
-  </si>
-  <si>
-    <t>U3</t>
-  </si>
-  <si>
-    <t>Blue-Pill</t>
-  </si>
-  <si>
     <t>U5</t>
   </si>
   <si>
@@ -316,9 +247,6 @@
     <t>C861535</t>
   </si>
   <si>
-    <t>R6</t>
-  </si>
-  <si>
     <t>R3</t>
   </si>
   <si>
@@ -335,6 +263,27 @@
   </si>
   <si>
     <t>C88185</t>
+  </si>
+  <si>
+    <t>D2, D3</t>
+  </si>
+  <si>
+    <t>R4, R7</t>
+  </si>
+  <si>
+    <t>R5, R9</t>
+  </si>
+  <si>
+    <t>R8, R10</t>
+  </si>
+  <si>
+    <t>1k</t>
+  </si>
+  <si>
+    <t>C14676</t>
+  </si>
+  <si>
+    <t>C2, C3, C4</t>
   </si>
 </sst>
 </file>
@@ -358,7 +307,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -366,12 +315,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -706,18 +669,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8748931B-0B37-431B-B398-955FDB268A91}">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.77734375" customWidth="1"/>
     <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="44.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.109375" customWidth="1"/>
+    <col min="8" max="8" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -726,12 +691,12 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -740,37 +705,55 @@
         <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
       <c r="D3" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
         <v>6</v>
       </c>
-      <c r="C4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
         <v>8</v>
@@ -779,320 +762,324 @@
         <v>9</v>
       </c>
       <c r="D5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" t="s">
+        <v>70</v>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" t="s">
+        <v>68</v>
+      </c>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s">
         <v>73</v>
       </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="C13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" t="s">
+        <v>76</v>
+      </c>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" t="s">
+        <v>56</v>
+      </c>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" t="s">
+        <v>57</v>
+      </c>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" t="s">
+        <v>58</v>
+      </c>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" t="s">
+        <v>59</v>
+      </c>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>15</v>
       </c>
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>90</v>
-      </c>
-      <c r="B11" t="s">
-        <v>91</v>
-      </c>
-      <c r="C11" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>86</v>
-      </c>
-      <c r="B13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>93</v>
-      </c>
-      <c r="B14" t="s">
-        <v>89</v>
-      </c>
-      <c r="C14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D14" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" t="s">
-        <v>88</v>
-      </c>
-      <c r="C15" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>34</v>
-      </c>
-      <c r="B16" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="B20" t="s">
         <v>37</v>
-      </c>
-      <c r="C18" t="s">
-        <v>38</v>
-      </c>
-      <c r="D18" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>41</v>
-      </c>
-      <c r="B19" t="s">
-        <v>40</v>
-      </c>
-      <c r="C19" t="s">
-        <v>38</v>
-      </c>
-      <c r="D19" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20" t="s">
-        <v>42</v>
       </c>
       <c r="C20" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D20" t="s">
+        <v>62</v>
+      </c>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C21" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>49</v>
-      </c>
-      <c r="B22" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" t="s">
-        <v>48</v>
-      </c>
-      <c r="D22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>51</v>
-      </c>
-      <c r="B23" t="s">
-        <v>50</v>
-      </c>
-      <c r="C23" t="s">
-        <v>48</v>
-      </c>
-      <c r="D23" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" t="s">
-        <v>52</v>
-      </c>
-      <c r="C24" t="s">
-        <v>48</v>
-      </c>
-      <c r="D24" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25" t="s">
-        <v>54</v>
-      </c>
-      <c r="C25" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>21</v>
-      </c>
-      <c r="B26" t="s">
-        <v>56</v>
-      </c>
-      <c r="C26" t="s">
-        <v>57</v>
-      </c>
-      <c r="D26" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>21</v>
-      </c>
-      <c r="B27" t="s">
-        <v>58</v>
-      </c>
-      <c r="C27" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>21</v>
-      </c>
-      <c r="B28" t="s">
-        <v>60</v>
-      </c>
-      <c r="C28" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>64</v>
-      </c>
-      <c r="B29" t="s">
-        <v>62</v>
-      </c>
-      <c r="C29" t="s">
-        <v>63</v>
-      </c>
-      <c r="D29" t="s">
-        <v>84</v>
-      </c>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added status LEDs to the DAQ board
</commit_message>
<xml_diff>
--- a/PCB/DAQBoardFront/JLCPCB Docs/BOM_DAQ.xlsx
+++ b/PCB/DAQBoardFront/JLCPCB Docs/BOM_DAQ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4a56d338d63da0fa/Desktop/CFR-2027/PCB/DAQBoardFront/JLCPCB Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="80" documentId="8_{672BEF6D-422F-477B-B486-B83020C6D7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EF2B4F8-5DBA-4DC7-9FF7-409359123BDF}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="8_{672BEF6D-422F-477B-B486-B83020C6D7F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E44F33A9-4696-4181-A18D-A29DB592FF2D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{93B5DAD3-BF6B-4E2E-A13F-1D74895200EB}"/>
   </bookViews>
@@ -274,9 +274,6 @@
     <t>R5, R9</t>
   </si>
   <si>
-    <t>R8, R10</t>
-  </si>
-  <si>
     <t>1k</t>
   </si>
   <si>
@@ -284,6 +281,9 @@
   </si>
   <si>
     <t>C2, C3, C4</t>
+  </si>
+  <si>
+    <t>R8, R10, R20, R21</t>
   </si>
 </sst>
 </file>
@@ -330,11 +330,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -669,7 +667,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8748931B-0B37-431B-B398-955FDB268A91}">
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.77734375" customWidth="1"/>
@@ -680,7 +678,7 @@
     <col min="9" max="9" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>42</v>
       </c>
@@ -694,7 +692,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -707,18 +705,13 @@
       <c r="D2" t="s">
         <v>45</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
@@ -726,13 +719,8 @@
       <c r="D3" t="s">
         <v>47</v>
       </c>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -745,13 +733,8 @@
       <c r="D4" t="s">
         <v>48</v>
       </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -764,13 +747,8 @@
       <c r="D5" t="s">
         <v>49</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -783,13 +761,8 @@
       <c r="D6" t="s">
         <v>51</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -802,13 +775,8 @@
       <c r="D7" t="s">
         <v>52</v>
       </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>66</v>
       </c>
@@ -821,13 +789,8 @@
       <c r="D8" t="s">
         <v>70</v>
       </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -840,13 +803,8 @@
       <c r="D9" t="s">
         <v>53</v>
       </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>63</v>
       </c>
@@ -859,13 +817,8 @@
       <c r="D10" t="s">
         <v>64</v>
       </c>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>69</v>
       </c>
@@ -878,17 +831,12 @@
       <c r="D11" t="s">
         <v>68</v>
       </c>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
         <v>72</v>
       </c>
       <c r="C12" t="s">
@@ -897,13 +845,8 @@
       <c r="D12" t="s">
         <v>54</v>
       </c>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -916,32 +859,22 @@
       <c r="D13" t="s">
         <v>55</v>
       </c>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B14" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s">
         <v>21</v>
       </c>
       <c r="D14" t="s">
-        <v>76</v>
-      </c>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -954,13 +887,8 @@
       <c r="D15" t="s">
         <v>56</v>
       </c>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -973,13 +901,8 @@
       <c r="D16" t="s">
         <v>57</v>
       </c>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -992,13 +915,8 @@
       <c r="D17" t="s">
         <v>58</v>
       </c>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -1011,13 +929,8 @@
       <c r="D18" t="s">
         <v>59</v>
       </c>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -1030,13 +943,8 @@
       <c r="D19" t="s">
         <v>60</v>
       </c>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>15</v>
       </c>
@@ -1049,13 +957,8 @@
       <c r="D20" t="s">
         <v>62</v>
       </c>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>41</v>
       </c>
@@ -1068,18 +971,6 @@
       <c r="D21" t="s">
         <v>61</v>
       </c>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>